<commit_message>
Added Code and report file
</commit_message>
<xml_diff>
--- a/testdata/login_data.xlsx
+++ b/testdata/login_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\Projects\Python Projects\capstone project\Parabank_automation\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5498B213-16FA-4E4F-8988-5A19D9502450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8787A453-3BA6-4C95-8F83-59A77CC9BA0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{27AFBE21-7BC4-4F1A-AB3C-1E51A80B585C}"/>
   </bookViews>
@@ -33,7 +33,7 @@
     <t>password</t>
   </si>
   <si>
-    <t>admin123</t>
+    <t>admin1234</t>
   </si>
 </sst>
 </file>

</xml_diff>